<commit_message>
Implemented several tab order and button color changes.
</commit_message>
<xml_diff>
--- a/.deploy/frontend-iis/templates/Bulk Upload Template.xlsx
+++ b/.deploy/frontend-iis/templates/Bulk Upload Template.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Development\Source\RPG Collection Navigator\frontend\public\templates\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f37c787087ac718/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6468A964-E9F0-4A6E-9E68-ED5B368C1E7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{739C80CC-CE39-4C57-B48D-26F4E2EFCDE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2475" yWindow="3585" windowWidth="28260" windowHeight="15990" xr2:uid="{2FC99663-8B02-44A8-96B9-B2E56A19E978}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="38610" windowHeight="20985" xr2:uid="{2FC99663-8B02-44A8-96B9-B2E56A19E978}"/>
   </bookViews>
   <sheets>
-    <sheet name="TestBulkUploadFile" sheetId="1" r:id="rId1"/>
+    <sheet name="Bulk Upload File" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>Publisher</t>
   </si>
@@ -41,6 +41,15 @@
   </si>
   <si>
     <t>Release Date</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>Is Physical</t>
+  </si>
+  <si>
+    <t>Is Digital</t>
   </si>
 </sst>
 </file>
@@ -902,19 +911,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F05FEC1-DF93-4DCD-980C-60C89C62D5CC}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.42578125" customWidth="1"/>
+    <col min="5" max="5" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -925,16 +935,25 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>